<commit_message>
Debugging formula excel template and XLOOKUP AND VLOOKUP
</commit_message>
<xml_diff>
--- a/2. Formula Excel Template.xlsx
+++ b/2. Formula Excel Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\All\codings\Data analytics\EXCELL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74807E83-8E89-4203-A50A-7866A5E8EEA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5505803-9D97-4042-AF89-3536CB30F476}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="4" xr2:uid="{47981922-77C5-4EC3-A76E-98D6CE997DC2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="5" activeTab="10" xr2:uid="{47981922-77C5-4EC3-A76E-98D6CE997DC2}"/>
   </bookViews>
   <sheets>
     <sheet name="Max-Min" sheetId="9" r:id="rId1"/>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="88">
   <si>
     <t>FirstName</t>
   </si>
@@ -1021,7 +1021,7 @@
   <sheetPr>
     <tabColor theme="9"/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="10.42578125" customWidth="1"/>
@@ -1030,9 +1030,10 @@
     <col min="8" max="8" width="14.28515625" customWidth="1"/>
     <col min="9" max="9" width="14.7109375" customWidth="1"/>
     <col min="10" max="10" width="22" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="27" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>20</v>
       </c>
@@ -1063,8 +1064,11 @@
       <c r="J1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1001</v>
       </c>
@@ -1092,8 +1096,16 @@
       <c r="I2" s="1">
         <v>42253</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J2" t="str" cm="1">
+        <f t="array" ref="J2:J10">CONCATENATE(B2:B10, " ", C2:C10)</f>
+        <v>Jim Halpert</v>
+      </c>
+      <c r="K2" t="str" cm="1">
+        <f t="array" ref="K2:K10">CONCATENATE(B2:B10,C2:C10,"@gmail.com")</f>
+        <v>JimHalpert@gmail.com</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1002</v>
       </c>
@@ -1121,8 +1133,14 @@
       <c r="I3" s="1">
         <v>42287</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J3" t="str">
+        <v>Pam Beasley</v>
+      </c>
+      <c r="K3" t="str">
+        <v>PamBeasley@gmail.com</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1003</v>
       </c>
@@ -1150,8 +1168,14 @@
       <c r="I4" s="1">
         <v>42986</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J4" t="str">
+        <v>Dwight Schrute</v>
+      </c>
+      <c r="K4" t="str">
+        <v>DwightSchrute@gmail.com</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1004</v>
       </c>
@@ -1179,8 +1203,14 @@
       <c r="I5" s="1">
         <v>42341</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J5" t="str">
+        <v>Angela Martin</v>
+      </c>
+      <c r="K5" t="str">
+        <v>AngelaMartin@gmail.com</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1005</v>
       </c>
@@ -1208,8 +1238,14 @@
       <c r="I6" s="1">
         <v>42977</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J6" t="str">
+        <v>Toby Flenderson</v>
+      </c>
+      <c r="K6" t="str">
+        <v>TobyFlenderson@gmail.com</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1006</v>
       </c>
@@ -1237,8 +1273,14 @@
       <c r="I7" s="1">
         <v>41528</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J7" t="str">
+        <v>Michael Scott</v>
+      </c>
+      <c r="K7" t="str">
+        <v>MichaelScott@gmail.com</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1007</v>
       </c>
@@ -1266,8 +1308,14 @@
       <c r="I8" s="1">
         <v>41551</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J8" t="str">
+        <v>Meredith Palmer</v>
+      </c>
+      <c r="K8" t="str">
+        <v>MeredithPalmer@gmail.com</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1008</v>
       </c>
@@ -1295,8 +1343,14 @@
       <c r="I9" s="1">
         <v>42116</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J9" t="str">
+        <v>Stanley Hudson</v>
+      </c>
+      <c r="K9" t="str">
+        <v>StanleyHudson@gmail.com</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1009</v>
       </c>
@@ -1324,14 +1378,20 @@
       <c r="I10" s="1">
         <v>40800</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J10" t="str">
+        <v>Kevin Malone</v>
+      </c>
+      <c r="K10" t="str">
+        <v>KevinMalone@gmail.com</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="H11" t="str">
         <f t="shared" ref="H11:H12" si="0">CONCATENATE(B11," ",C11)</f>
         <v xml:space="preserve"> </v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="H12" t="str">
         <f t="shared" si="0"/>
         <v xml:space="preserve"> </v>
@@ -1417,6 +1477,14 @@
       <c r="I2" s="2" t="s">
         <v>56</v>
       </c>
+      <c r="J2" cm="1">
+        <f t="array" ref="J2:J10">_xlfn.DAYS(I2:I10,H2:H10)</f>
+        <v>5056</v>
+      </c>
+      <c r="K2">
+        <f>NETWORKDAYS(H2,I2)</f>
+        <v>3611</v>
+      </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
@@ -1446,6 +1514,13 @@
       <c r="I3" s="2" t="s">
         <v>57</v>
       </c>
+      <c r="J3">
+        <v>5851</v>
+      </c>
+      <c r="K3">
+        <f t="shared" ref="K3:K10" si="0">NETWORKDAYS(H3,I3)</f>
+        <v>4180</v>
+      </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
@@ -1475,6 +1550,13 @@
       <c r="I4" s="2" t="s">
         <v>58</v>
       </c>
+      <c r="J4">
+        <v>6275</v>
+      </c>
+      <c r="K4">
+        <f t="shared" si="0"/>
+        <v>4484</v>
+      </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
@@ -1504,6 +1586,13 @@
       <c r="I5" s="2" t="s">
         <v>59</v>
       </c>
+      <c r="J5">
+        <v>5811</v>
+      </c>
+      <c r="K5">
+        <f t="shared" si="0"/>
+        <v>4152</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
@@ -1533,6 +1622,13 @@
       <c r="I6" s="2" t="s">
         <v>60</v>
       </c>
+      <c r="J6">
+        <v>5960</v>
+      </c>
+      <c r="K6">
+        <f t="shared" si="0"/>
+        <v>4258</v>
+      </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
@@ -1562,6 +1658,13 @@
       <c r="I7" s="2" t="s">
         <v>61</v>
       </c>
+      <c r="J7">
+        <v>4511</v>
+      </c>
+      <c r="K7">
+        <f t="shared" si="0"/>
+        <v>3223</v>
+      </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8">
@@ -1591,6 +1694,13 @@
       <c r="I8" s="2" t="s">
         <v>61</v>
       </c>
+      <c r="J8">
+        <v>3595</v>
+      </c>
+      <c r="K8">
+        <f t="shared" si="0"/>
+        <v>2568</v>
+      </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9">
@@ -1620,6 +1730,13 @@
       <c r="I9" s="2" t="s">
         <v>62</v>
       </c>
+      <c r="J9">
+        <v>4700</v>
+      </c>
+      <c r="K9">
+        <f t="shared" si="0"/>
+        <v>3358</v>
+      </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10">
@@ -1648,6 +1765,13 @@
       </c>
       <c r="I10" s="2" t="s">
         <v>62</v>
+      </c>
+      <c r="J10">
+        <v>4273</v>
+      </c>
+      <c r="K10">
+        <f t="shared" si="0"/>
+        <v>3053</v>
       </c>
     </row>
   </sheetData>
@@ -3254,6 +3378,10 @@
       <c r="I2" s="1">
         <v>42253</v>
       </c>
+      <c r="J2" t="str" cm="1">
+        <f t="array" ref="J2:J10">TRIM(C2:C10)</f>
+        <v>Halpert</v>
+      </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
@@ -3283,6 +3411,9 @@
       <c r="I3" s="1">
         <v>42287</v>
       </c>
+      <c r="J3" t="str">
+        <v>Beasley</v>
+      </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
@@ -3312,6 +3443,9 @@
       <c r="I4" s="1">
         <v>42986</v>
       </c>
+      <c r="J4" t="str">
+        <v>Schrute</v>
+      </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
@@ -3341,6 +3475,9 @@
       <c r="I5" s="1">
         <v>42341</v>
       </c>
+      <c r="J5" t="str">
+        <v>Martin</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
@@ -3370,6 +3507,9 @@
       <c r="I6" s="1">
         <v>42977</v>
       </c>
+      <c r="J6" t="str">
+        <v>Flenderson</v>
+      </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
@@ -3399,6 +3539,9 @@
       <c r="I7" s="1">
         <v>41528</v>
       </c>
+      <c r="J7" t="str">
+        <v>Scott</v>
+      </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8">
@@ -3428,6 +3571,9 @@
       <c r="I8" s="1">
         <v>41551</v>
       </c>
+      <c r="J8" t="str">
+        <v>Palmer</v>
+      </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9">
@@ -3457,6 +3603,9 @@
       <c r="I9" s="1">
         <v>42116</v>
       </c>
+      <c r="J9" t="str">
+        <v>Hudson</v>
+      </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10">
@@ -3485,6 +3634,9 @@
       </c>
       <c r="I10" s="1">
         <v>40800</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Malone</v>
       </c>
     </row>
   </sheetData>
@@ -3570,6 +3722,18 @@
       <c r="I2" s="2" t="s">
         <v>56</v>
       </c>
+      <c r="J2" t="str" cm="1">
+        <f t="array" ref="J2:J10">SUBSTITUTE(H2:H10,"/","-",1)</f>
+        <v>11-2/2001</v>
+      </c>
+      <c r="K2" t="str" cm="1">
+        <f t="array" ref="K2:K10">SUBSTITUTE(H2:H10,"/","-",2)</f>
+        <v>11/2-2001</v>
+      </c>
+      <c r="L2" t="str" cm="1">
+        <f t="array" ref="L2:L10">SUBSTITUTE(H2:H10,"/","-")</f>
+        <v>11-2-2001</v>
+      </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3">
@@ -3599,6 +3763,15 @@
       <c r="I3" s="2" t="s">
         <v>57</v>
       </c>
+      <c r="J3" t="str">
+        <v>10-3/1999</v>
+      </c>
+      <c r="K3" t="str">
+        <v>10/3-1999</v>
+      </c>
+      <c r="L3" t="str">
+        <v>10-3-1999</v>
+      </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4">
@@ -3628,6 +3801,15 @@
       <c r="I4" s="2" t="s">
         <v>58</v>
       </c>
+      <c r="J4" t="str">
+        <v>7-4/2000</v>
+      </c>
+      <c r="K4" t="str">
+        <v>7/4-2000</v>
+      </c>
+      <c r="L4" t="str">
+        <v>7-4-2000</v>
+      </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5">
@@ -3657,6 +3839,15 @@
       <c r="I5" s="2" t="s">
         <v>59</v>
       </c>
+      <c r="J5" t="str">
+        <v>1-5/2000</v>
+      </c>
+      <c r="K5" t="str">
+        <v>1/5-2000</v>
+      </c>
+      <c r="L5" t="str">
+        <v>1-5-2000</v>
+      </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6">
@@ -3686,6 +3877,15 @@
       <c r="I6" s="2" t="s">
         <v>60</v>
       </c>
+      <c r="J6" t="str">
+        <v>5-6/2001</v>
+      </c>
+      <c r="K6" t="str">
+        <v>5/6-2001</v>
+      </c>
+      <c r="L6" t="str">
+        <v>5-6-2001</v>
+      </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7">
@@ -3715,6 +3915,15 @@
       <c r="I7" s="2" t="s">
         <v>61</v>
       </c>
+      <c r="J7" t="str">
+        <v>5-6/2001</v>
+      </c>
+      <c r="K7" t="str">
+        <v>5/6-2001</v>
+      </c>
+      <c r="L7" t="str">
+        <v>5-6-2001</v>
+      </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8">
@@ -3744,6 +3953,15 @@
       <c r="I8" s="2" t="s">
         <v>61</v>
       </c>
+      <c r="J8" t="str">
+        <v>11-8/2003</v>
+      </c>
+      <c r="K8" t="str">
+        <v>11/8-2003</v>
+      </c>
+      <c r="L8" t="str">
+        <v>11-8-2003</v>
+      </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9">
@@ -3773,6 +3991,15 @@
       <c r="I9" s="2" t="s">
         <v>62</v>
       </c>
+      <c r="J9" t="str">
+        <v>6-9/2002</v>
+      </c>
+      <c r="K9" t="str">
+        <v>6/9-2002</v>
+      </c>
+      <c r="L9" t="str">
+        <v>6-9-2002</v>
+      </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10">
@@ -3801,6 +4028,15 @@
       </c>
       <c r="I10" s="2" t="s">
         <v>62</v>
+      </c>
+      <c r="J10" t="str">
+        <v>8-10/2003</v>
+      </c>
+      <c r="K10" t="str">
+        <v>8/10-2003</v>
+      </c>
+      <c r="L10" t="str">
+        <v>8-10-2003</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
@@ -3918,6 +4154,18 @@
       </c>
       <c r="I2" s="1">
         <v>42253</v>
+      </c>
+      <c r="J2">
+        <f>SUM(G2:G10)</f>
+        <v>437000</v>
+      </c>
+      <c r="K2">
+        <f>SUMIF(G2:G10,"&gt;50000")</f>
+        <v>128000</v>
+      </c>
+      <c r="L2">
+        <f>SUMIFS(G2:G10,E2:E10,"Female",D2:D10,"&gt;30")</f>
+        <v>88000</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -4235,6 +4483,18 @@
       <c r="I2" s="1">
         <v>42253</v>
       </c>
+      <c r="J2">
+        <f>COUNT(D2:D10)</f>
+        <v>9</v>
+      </c>
+      <c r="K2">
+        <f>COUNTIF(G2:G10,"&gt;50000")</f>
+        <v>2</v>
+      </c>
+      <c r="L2">
+        <f>COUNTIFS(D2:D10,"&gt;30",G2:G10,"50000")</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3">
@@ -4263,6 +4523,14 @@
       </c>
       <c r="I3" s="1">
         <v>42287</v>
+      </c>
+      <c r="J3">
+        <f>COUNT(A4:I4)</f>
+        <v>5</v>
+      </c>
+      <c r="K3">
+        <f>COUNTIF(D2:D10,"&gt;32")</f>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">

</xml_diff>